<commit_message>
Update department code mapping
</commit_message>
<xml_diff>
--- a/data/11505/系所經費代碼與中文名稱對照表.xlsx
+++ b/data/11505/系所經費代碼與中文名稱對照表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\IR大數據分析組\IR-躍升相關\經費收支明細\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC8DD0A-16FF-4247-8365-BF14617CED58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19E43302-C45D-4D91-B716-8129F875AEB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A410AB86-5814-4FCF-ADFA-7EA48B0B568D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A410AB86-5814-4FCF-ADFA-7EA48B0B568D}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="117">
   <si>
     <r>
       <rPr>
@@ -1102,6 +1102,10 @@
       </rPr>
       <t>)</t>
     </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>UT02</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -1401,6 +1405,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1417,12 +1427,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1739,7 +1743,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D452D504-C59B-4FEE-9796-EA0E20A0674F}">
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.125" bestFit="1" customWidth="1"/>
@@ -1748,20 +1752,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="17" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12"/>
-      <c r="B2" s="14"/>
-      <c r="C2" s="16"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="18"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -1836,7 +1840,7 @@
       <c r="B9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="11" t="s">
         <v>107</v>
       </c>
     </row>
@@ -1943,7 +1947,7 @@
       <c r="A19" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="12" t="s">
         <v>115</v>
       </c>
       <c r="C19" s="6" t="s">
@@ -2034,7 +2038,7 @@
       <c r="B27" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="17" t="s">
+      <c r="C27" s="11" t="s">
         <v>113</v>
       </c>
       <c r="D27" t="s">
@@ -2081,7 +2085,7 @@
       <c r="B31" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C31" s="17" t="s">
+      <c r="C31" s="11" t="s">
         <v>112</v>
       </c>
       <c r="D31" t="s">
@@ -2101,24 +2105,27 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>66</v>
+        <v>63</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="D33" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -2126,21 +2133,21 @@
         <v>3</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -2148,32 +2155,32 @@
         <v>20</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -2181,10 +2188,10 @@
         <v>20</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -2194,80 +2201,80 @@
       <c r="B41" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C41" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="D41" t="s">
-        <v>109</v>
+      <c r="C41" s="6" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>82</v>
+        <v>79</v>
+      </c>
+      <c r="C42" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="D42" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B43" s="18" t="s">
-        <v>111</v>
-      </c>
-      <c r="C43" s="17" t="s">
-        <v>110</v>
-      </c>
-      <c r="D43" t="s">
-        <v>109</v>
+      <c r="B43" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>85</v>
+        <v>17</v>
+      </c>
+      <c r="B44" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="C44" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="D44" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
-        <v>42</v>
+        <v>83</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -2275,21 +2282,21 @@
         <v>83</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -2297,10 +2304,10 @@
         <v>94</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -2308,42 +2315,53 @@
         <v>94</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>6</v>
+        <v>94</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B53" s="5" t="s">
+      <c r="B54" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C53" s="6" t="s">
+      <c r="C54" s="6" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="8" t="s">
+    <row r="55" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B54" s="9" t="s">
+      <c r="B55" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="C54" s="10" t="s">
+      <c r="C55" s="10" t="s">
         <v>106</v>
       </c>
     </row>

</xml_diff>